<commit_message>
Agregar funcionalidad para crear y recomendar funciones entre columnas en la ventana principal. Se implementa un botón que permite al usuario generar una función utilizando IA, así como un campo editable para modificar la función sugerida. Además, se actualiza el diálogo de agrupación cualitativa para manejar respuestas de agrupación de manera más estructurada. Se mejora la integración con la API de Gemini para obtener sugerencias de funciones y se añaden validaciones para asegurar la correcta ejecución de estas nuevas características.
</commit_message>
<xml_diff>
--- a/student_health_data_rows.xlsx
+++ b/student_health_data_rows.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ZLostTK\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ZLostTK\Downloads\project-bolt-sb1-flngyft9\project\PROGRAMA BIEN HECHO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19D83DAF-D99B-4FB5-8C52-7E7C8A3A2CBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D85620C2-3EA2-43F2-B908-595D8FF490EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{67CCEE16-EC59-4560-935F-9241ACC138B0}"/>
   </bookViews>
@@ -3050,7 +3050,7 @@
         <v>11</v>
       </c>
       <c r="F54">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G54">
         <v>65</v>
@@ -3114,7 +3114,7 @@
         <v>43</v>
       </c>
       <c r="F56">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G56">
         <v>51</v>
@@ -3146,7 +3146,7 @@
         <v>82</v>
       </c>
       <c r="F57">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G57">
         <v>75</v>
@@ -3274,7 +3274,7 @@
         <v>11</v>
       </c>
       <c r="F61">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G61">
         <v>52</v>
@@ -3338,7 +3338,7 @@
         <v>43</v>
       </c>
       <c r="F63">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G63">
         <v>59</v>
@@ -3370,7 +3370,7 @@
         <v>43</v>
       </c>
       <c r="F64">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G64">
         <v>79</v>
@@ -3402,7 +3402,7 @@
         <v>11</v>
       </c>
       <c r="F65">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G65">
         <v>62</v>
@@ -3562,7 +3562,7 @@
         <v>43</v>
       </c>
       <c r="F70">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G70">
         <v>77</v>

</xml_diff>

<commit_message>
Actualizar `requirements.txt` para incluir nuevas dependencias: `sympy` y `google-genai`. Además, se actualiza el archivo `student_health_data_rows.xlsx` con cambios binarios.
</commit_message>
<xml_diff>
--- a/student_health_data_rows.xlsx
+++ b/student_health_data_rows.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ZLostTK\Downloads\project-bolt-sb1-flngyft9\project\PROGRAMA BIEN HECHO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D85620C2-3EA2-43F2-B908-595D8FF490EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFD9A0D4-CAEE-4B8D-82CC-95645508610B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{67CCEE16-EC59-4560-935F-9241ACC138B0}"/>
+    <workbookView xWindow="7200" yWindow="4170" windowWidth="21600" windowHeight="11385" xr2:uid="{67CCEE16-EC59-4560-935F-9241ACC138B0}"/>
   </bookViews>
   <sheets>
     <sheet name="student_health_data_rows" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="153">
   <si>
     <t>id</t>
   </si>
@@ -83,9 +83,6 @@
   </si>
   <si>
     <t>2025-05-10 03:37:14.948204+00</t>
-  </si>
-  <si>
-    <t>A</t>
   </si>
   <si>
     <t>2025-05-10 03:39:33.302005+00</t>
@@ -1377,7 +1374,7 @@
         <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D2">
         <v>4</v>
@@ -1441,7 +1438,7 @@
         <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D4">
         <v>4</v>
@@ -1473,7 +1470,7 @@
         <v>16</v>
       </c>
       <c r="C5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D5">
         <v>4</v>
@@ -1505,7 +1502,7 @@
         <v>18</v>
       </c>
       <c r="C6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D6">
         <v>4</v>
@@ -1537,7 +1534,7 @@
         <v>19</v>
       </c>
       <c r="C7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D7">
         <v>4</v>
@@ -1569,13 +1566,13 @@
         <v>20</v>
       </c>
       <c r="C8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D8">
         <v>4</v>
       </c>
       <c r="E8" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F8">
         <v>16</v>
@@ -1598,16 +1595,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" t="s">
+        <v>111</v>
+      </c>
+      <c r="D9">
+        <v>4</v>
+      </c>
+      <c r="E9" t="s">
         <v>22</v>
-      </c>
-      <c r="C9" t="s">
-        <v>112</v>
-      </c>
-      <c r="D9">
-        <v>4</v>
-      </c>
-      <c r="E9" t="s">
-        <v>23</v>
       </c>
       <c r="F9">
         <v>16</v>
@@ -1630,16 +1627,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C10" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D10">
         <v>4</v>
       </c>
       <c r="E10" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F10">
         <v>17</v>
@@ -1662,16 +1659,16 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" t="s">
+        <v>113</v>
+      </c>
+      <c r="D11">
+        <v>4</v>
+      </c>
+      <c r="E11" t="s">
         <v>25</v>
-      </c>
-      <c r="C11" t="s">
-        <v>114</v>
-      </c>
-      <c r="D11">
-        <v>4</v>
-      </c>
-      <c r="E11" t="s">
-        <v>26</v>
       </c>
       <c r="F11">
         <v>16</v>
@@ -1694,16 +1691,16 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C12" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D12">
         <v>4</v>
       </c>
       <c r="E12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F12">
         <v>16</v>
@@ -1726,16 +1723,16 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C13" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D13">
         <v>4</v>
       </c>
       <c r="E13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F13">
         <v>17</v>
@@ -1758,16 +1755,16 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C14" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D14">
         <v>4</v>
       </c>
       <c r="E14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F14">
         <v>16</v>
@@ -1790,16 +1787,16 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C15" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D15">
         <v>2</v>
       </c>
       <c r="E15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F15">
         <v>15</v>
@@ -1822,10 +1819,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C16" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D16">
         <v>6</v>
@@ -1854,10 +1851,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C17" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D17">
         <v>6</v>
@@ -1886,7 +1883,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C18" t="s">
         <v>13</v>
@@ -1918,10 +1915,10 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C19" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D19">
         <v>6</v>
@@ -1950,10 +1947,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C20" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D20">
         <v>6</v>
@@ -1982,10 +1979,10 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C21" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D21">
         <v>6</v>
@@ -2014,10 +2011,10 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C22" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D22">
         <v>6</v>
@@ -2046,10 +2043,10 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C23" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D23">
         <v>6</v>
@@ -2078,16 +2075,16 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C24" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D24">
         <v>2</v>
       </c>
       <c r="E24" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F24">
         <v>15</v>
@@ -2110,16 +2107,16 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C25" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D25">
         <v>2</v>
       </c>
       <c r="E25" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F25">
         <v>16</v>
@@ -2142,16 +2139,16 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C26" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D26">
         <v>6</v>
       </c>
       <c r="E26" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F26">
         <v>18</v>
@@ -2174,16 +2171,16 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C27" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D27">
         <v>6</v>
       </c>
       <c r="E27" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F27">
         <v>17</v>
@@ -2206,16 +2203,16 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C28" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D28">
         <v>6</v>
       </c>
       <c r="E28" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F28">
         <v>17</v>
@@ -2238,16 +2235,16 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C29" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D29">
         <v>6</v>
       </c>
       <c r="E29" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F29">
         <v>18</v>
@@ -2270,16 +2267,16 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C30" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D30">
         <v>2</v>
       </c>
       <c r="E30" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F30">
         <v>15</v>
@@ -2302,16 +2299,16 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C31" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D31">
         <v>2</v>
       </c>
       <c r="E31" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F31">
         <v>15</v>
@@ -2334,16 +2331,16 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C32" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D32">
         <v>4</v>
       </c>
       <c r="E32" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F32">
         <v>16</v>
@@ -2366,16 +2363,16 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C33" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D33">
         <v>2</v>
       </c>
       <c r="E33" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F33">
         <v>15</v>
@@ -2398,16 +2395,16 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
+        <v>50</v>
+      </c>
+      <c r="C34" t="s">
         <v>51</v>
-      </c>
-      <c r="C34" t="s">
-        <v>52</v>
       </c>
       <c r="D34">
         <v>2</v>
       </c>
       <c r="E34" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F34">
         <v>15</v>
@@ -2430,16 +2427,16 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C35" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D35">
         <v>2</v>
       </c>
       <c r="E35" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F35">
         <v>15</v>
@@ -2462,16 +2459,16 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C36" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D36">
         <v>4</v>
       </c>
       <c r="E36" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F36">
         <v>17</v>
@@ -2494,10 +2491,10 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C37" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D37">
         <v>4</v>
@@ -2526,16 +2523,16 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C38" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D38">
         <v>4</v>
       </c>
       <c r="E38" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F38">
         <v>16</v>
@@ -2558,10 +2555,10 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C39" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D39">
         <v>4</v>
@@ -2590,10 +2587,10 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D40">
         <v>4</v>
@@ -2622,10 +2619,10 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C41" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D41">
         <v>4</v>
@@ -2654,16 +2651,16 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
+        <v>59</v>
+      </c>
+      <c r="C42" t="s">
         <v>60</v>
-      </c>
-      <c r="C42" t="s">
-        <v>61</v>
       </c>
       <c r="D42">
         <v>6</v>
       </c>
       <c r="E42" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F42">
         <v>18</v>
@@ -2686,16 +2683,16 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
+        <v>61</v>
+      </c>
+      <c r="C43" t="s">
         <v>62</v>
-      </c>
-      <c r="C43" t="s">
-        <v>63</v>
       </c>
       <c r="D43">
         <v>6</v>
       </c>
       <c r="E43" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F43">
         <v>17</v>
@@ -2718,16 +2715,16 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
+        <v>63</v>
+      </c>
+      <c r="C44" t="s">
         <v>64</v>
-      </c>
-      <c r="C44" t="s">
-        <v>65</v>
       </c>
       <c r="D44">
         <v>6</v>
       </c>
       <c r="E44" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F44">
         <v>17</v>
@@ -2750,16 +2747,16 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C45" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D45">
         <v>2</v>
       </c>
       <c r="E45" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F45">
         <v>16</v>
@@ -2782,10 +2779,10 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C46" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D46">
         <v>4</v>
@@ -2814,10 +2811,10 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C47" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D47">
         <v>4</v>
@@ -2846,16 +2843,16 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
+        <v>69</v>
+      </c>
+      <c r="C48" t="s">
         <v>70</v>
-      </c>
-      <c r="C48" t="s">
-        <v>71</v>
       </c>
       <c r="D48">
         <v>2</v>
       </c>
       <c r="E48" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F48">
         <v>15</v>
@@ -2878,16 +2875,16 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
+        <v>71</v>
+      </c>
+      <c r="C49" t="s">
         <v>72</v>
-      </c>
-      <c r="C49" t="s">
-        <v>73</v>
       </c>
       <c r="D49">
         <v>2</v>
       </c>
       <c r="E49" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F49">
         <v>16</v>
@@ -2910,16 +2907,16 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C50" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D50">
         <v>6</v>
       </c>
       <c r="E50" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F50">
         <v>17</v>
@@ -2942,10 +2939,10 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
+        <v>75</v>
+      </c>
+      <c r="C51" t="s">
         <v>76</v>
-      </c>
-      <c r="C51" t="s">
-        <v>77</v>
       </c>
       <c r="D51">
         <v>6</v>
@@ -2974,10 +2971,10 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
+        <v>77</v>
+      </c>
+      <c r="C52" t="s">
         <v>78</v>
-      </c>
-      <c r="C52" t="s">
-        <v>79</v>
       </c>
       <c r="D52">
         <v>6</v>
@@ -3006,10 +3003,10 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C53" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D53">
         <v>4</v>
@@ -3038,10 +3035,10 @@
         <v>53</v>
       </c>
       <c r="B54" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C54" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D54">
         <v>4</v>
@@ -3070,10 +3067,10 @@
         <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C55" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D55">
         <v>4</v>
@@ -3102,16 +3099,16 @@
         <v>55</v>
       </c>
       <c r="B56" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C56" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D56">
         <v>4</v>
       </c>
       <c r="E56" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F56">
         <v>17</v>
@@ -3134,16 +3131,16 @@
         <v>56</v>
       </c>
       <c r="B57" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C57" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D57">
         <v>2</v>
       </c>
       <c r="E57" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F57">
         <v>15</v>
@@ -3166,16 +3163,16 @@
         <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C58" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D58">
         <v>4</v>
       </c>
       <c r="E58" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F58">
         <v>16</v>
@@ -3198,10 +3195,10 @@
         <v>58</v>
       </c>
       <c r="B59" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C59" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D59">
         <v>2</v>
@@ -3230,10 +3227,10 @@
         <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C60" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D60">
         <v>4</v>
@@ -3262,10 +3259,10 @@
         <v>60</v>
       </c>
       <c r="B61" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C61" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D61">
         <v>2</v>
@@ -3294,16 +3291,16 @@
         <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C62" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D62">
         <v>4</v>
       </c>
       <c r="E62" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F62">
         <v>17</v>
@@ -3326,16 +3323,16 @@
         <v>62</v>
       </c>
       <c r="B63" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C63" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D63">
         <v>4</v>
       </c>
       <c r="E63" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F63">
         <v>17</v>
@@ -3358,16 +3355,16 @@
         <v>63</v>
       </c>
       <c r="B64" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C64" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D64">
         <v>4</v>
       </c>
       <c r="E64" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F64">
         <v>17</v>
@@ -3390,10 +3387,10 @@
         <v>64</v>
       </c>
       <c r="B65" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C65" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D65">
         <v>4</v>
@@ -3422,10 +3419,10 @@
         <v>65</v>
       </c>
       <c r="B66" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C66" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D66">
         <v>4</v>
@@ -3454,10 +3451,10 @@
         <v>66</v>
       </c>
       <c r="B67" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C67" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D67">
         <v>4</v>
@@ -3486,16 +3483,16 @@
         <v>67</v>
       </c>
       <c r="B68" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C68" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D68">
         <v>2</v>
       </c>
       <c r="E68" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F68">
         <v>16</v>
@@ -3518,16 +3515,16 @@
         <v>68</v>
       </c>
       <c r="B69" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C69" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D69">
         <v>6</v>
       </c>
       <c r="E69" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F69">
         <v>18</v>
@@ -3550,16 +3547,16 @@
         <v>69</v>
       </c>
       <c r="B70" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C70" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D70">
         <v>4</v>
       </c>
       <c r="E70" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F70">
         <v>17</v>
@@ -3582,10 +3579,10 @@
         <v>70</v>
       </c>
       <c r="B71" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C71" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D71">
         <v>4</v>

</xml_diff>